<commit_message>
Updated import export to v4.1.1
1. Updated import and export
2. Updated Data Import Template and Sample Data File
</commit_message>
<xml_diff>
--- a/downloads/TUVAT CVS Training - Data Import Template.xlsx
+++ b/downloads/TUVAT CVS Training - Data Import Template.xlsx
@@ -1,22 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\verify-cert-training\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383E834C-CCEE-4660-A450-FA914CBC2181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740CC910-C029-41A4-8FE4-D138910A6D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>certificate_number</t>
   </si>
@@ -76,6 +85,12 @@
   </si>
   <si>
     <t>signatory_email</t>
+  </si>
+  <si>
+    <t>has_practical</t>
+  </si>
+  <si>
+    <t>is_refresher</t>
   </si>
 </sst>
 </file>
@@ -423,28 +438,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:T1"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.88671875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="1" width="18.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.85546875" style="2" customWidth="1"/>
+    <col min="15" max="15" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -452,51 +469,57 @@
         <v>14</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="1"/>
+      <c r="T1" s="1"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>

</xml_diff>